<commit_message>
Fixed inconsistency between grading and inter-rater computations + regenerated figures
</commit_message>
<xml_diff>
--- a/Automatic Bread Maker/Grading/1 stage/3-examples/Automatic-Bread-Maker_Grading_1-stage_2026-02-28_3-examples_CombinedHumanGradingVsClaude4.5SonnetAutoGrading_Claude4.5SonnetGeneration.xlsx
+++ b/Automatic Bread Maker/Grading/1 stage/3-examples/Automatic-Bread-Maker_Grading_1-stage_2026-02-28_3-examples_CombinedHumanGradingVsClaude4.5SonnetAutoGrading_Claude4.5SonnetGeneration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marc-antoinenadeau/Desktop/Evaluations 2/Automatic Bread Maker/Grading/1 stage/2026-02-28/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marc-antoinenadeau/Desktop/B.Eng Software Engineering /7th Semester/Capstone/Code/Evaluations/Automatic Bread Maker/Grading/1 stage/3-examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D998E64C-3BA4-B242-9E3A-0405406A5485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4167CB-AA33-3A4C-9A32-256A335F7DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Automatic Bread Maker" sheetId="1" r:id="rId1"/>
@@ -1115,24 +1115,30 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="23">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1304,39 +1310,39 @@
   </dxfs>
   <tableStyles count="7">
     <tableStyle name="Automatic Bread Maker-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="headerRow" dxfId="20"/>
-      <tableStyleElement type="firstRowStripe" dxfId="19"/>
-      <tableStyleElement type="secondRowStripe" dxfId="18"/>
+      <tableStyleElement type="headerRow" dxfId="22"/>
+      <tableStyleElement type="firstRowStripe" dxfId="21"/>
+      <tableStyleElement type="secondRowStripe" dxfId="20"/>
     </tableStyle>
     <tableStyle name="Human Grading-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="headerRow" dxfId="17"/>
-      <tableStyleElement type="firstRowStripe" dxfId="16"/>
-      <tableStyleElement type="secondRowStripe" dxfId="15"/>
+      <tableStyleElement type="headerRow" dxfId="19"/>
+      <tableStyleElement type="firstRowStripe" dxfId="18"/>
+      <tableStyleElement type="secondRowStripe" dxfId="17"/>
     </tableStyle>
     <tableStyle name="LLM Grading-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="headerRow" dxfId="14"/>
-      <tableStyleElement type="firstRowStripe" dxfId="13"/>
-      <tableStyleElement type="secondRowStripe" dxfId="12"/>
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="firstRowStripe" dxfId="15"/>
+      <tableStyleElement type="secondRowStripe" dxfId="14"/>
     </tableStyle>
     <tableStyle name="Metrics-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="firstRowStripe" dxfId="10"/>
-      <tableStyleElement type="secondRowStripe" dxfId="9"/>
+      <tableStyleElement type="headerRow" dxfId="13"/>
+      <tableStyleElement type="firstRowStripe" dxfId="12"/>
+      <tableStyleElement type="secondRowStripe" dxfId="11"/>
     </tableStyle>
     <tableStyle name="Metrics-style 2" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="headerRow" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="secondRowStripe" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="firstRowStripe" dxfId="9"/>
+      <tableStyleElement type="secondRowStripe" dxfId="8"/>
     </tableStyle>
     <tableStyle name="Inter-rater-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="firstRowStripe" dxfId="4"/>
-      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+      <tableStyleElement type="firstRowStripe" dxfId="6"/>
+      <tableStyleElement type="secondRowStripe" dxfId="5"/>
     </tableStyle>
     <tableStyle name="Weighted Cohens Kappa-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
-      <tableStyleElement type="headerRow" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="secondRowStripe" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="4"/>
+      <tableStyleElement type="firstRowStripe" dxfId="3"/>
+      <tableStyleElement type="secondRowStripe" dxfId="2"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1403,12 +1409,20 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table_6" displayName="Table_6" ref="A1:D54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table_6" displayName="Table_6" ref="A1:D56">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Type"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Element"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Human"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="LLM"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Type" dataDxfId="1">
+      <calculatedColumnFormula>'Human Grading'!A2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Element" dataDxfId="0">
+      <calculatedColumnFormula>'Human Grading'!B2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Human">
+      <calculatedColumnFormula>'Human Grading'!C2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="LLM">
+      <calculatedColumnFormula>'LLM Grading'!C2</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Inter-rater-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17772,16 +17786,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="70" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
       <c r="J1" s="36" t="s">
         <v>115</v>
       </c>
@@ -18089,16 +18103,16 @@
     </row>
     <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="67" t="s">
+      <c r="A12" s="70" t="s">
         <v>165</v>
       </c>
-      <c r="B12" s="68"/>
-      <c r="C12" s="68"/>
-      <c r="D12" s="68"/>
-      <c r="E12" s="68"/>
-      <c r="F12" s="68"/>
-      <c r="G12" s="68"/>
-      <c r="H12" s="68"/>
+      <c r="B12" s="71"/>
+      <c r="C12" s="71"/>
+      <c r="D12" s="71"/>
+      <c r="E12" s="71"/>
+      <c r="F12" s="71"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="71"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="37" t="s">
@@ -19412,33 +19426,33 @@
       <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="73" t="s">
+      <c r="C1" s="67" t="s">
         <v>166</v>
       </c>
-      <c r="D1" s="73" t="s">
+      <c r="D1" s="67" t="s">
         <v>60</v>
       </c>
       <c r="E1" s="44"/>
-      <c r="F1" s="69" t="s">
+      <c r="F1" s="68" t="s">
         <v>128</v>
       </c>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="L1" s="71" t="s">
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="L1" s="72" t="s">
         <v>129</v>
       </c>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="str">
-        <f>'Human Grading'!A3</f>
+        <f>'Human Grading'!A2</f>
         <v>State</v>
       </c>
       <c r="B2" s="5" t="str">
-        <f>'Human Grading'!B3</f>
-        <v>Off</v>
+        <f>'Human Grading'!B2</f>
+        <v>Initial state (→ Off)</v>
       </c>
       <c r="C2" s="5">
         <f>'Human Grading'!C2</f>
@@ -19477,12 +19491,12 @@
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="5" t="str">
-        <f>'Human Grading'!A4</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A3</f>
+        <v>State</v>
       </c>
       <c r="B3" s="5" t="str">
-        <f>'Human Grading'!B4</f>
-        <v>on (Off ⇒ On)</v>
+        <f>'Human Grading'!B3</f>
+        <v>Off</v>
       </c>
       <c r="C3" s="5">
         <f>'Human Grading'!C3</f>
@@ -19497,28 +19511,28 @@
         <v>0</v>
       </c>
       <c r="G3" s="52">
-        <f>COUNTIFS($C$2:$C$91, $F3, $D$2:$D$91, G$2)</f>
-        <v>12</v>
+        <f>COUNTIFS($C$2:$C$93, $F3, $D$2:$D$93, G$2)</f>
+        <v>14</v>
       </c>
       <c r="H3" s="53">
-        <f>COUNTIFS($C$2:$C$47, $F3, $D$2:$D$47, H$2)</f>
+        <f>COUNTIFS($C$2:$C$49, $F3, $D$2:$D$49, H$2)</f>
         <v>0</v>
       </c>
       <c r="I3" s="54">
-        <f>COUNTIFS($C$2:$C$47, $F3, $D$2:$D$47, I$2)+MAX(D48-C48,0)+MAX(D49-C49,0)+MAX(D50-C50,0)+MAX(D51-C51,0)+MAX(D52-C52,0)+MAX(D53-C53,0)+MAX(D54-C54,0)</f>
+        <f>COUNTIFS($C$2:$C$49, $F3, $D$2:$D$49, I$2)+MAX(D50-C50,0)+MAX(D51-C51,0)+MAX(D52-C52,0)+MAX(D53-C53,0)+MAX(D54-C54,0)+MAX(D55-C55,0)+MAX(D56-C56,0)</f>
         <v>1</v>
       </c>
       <c r="J3" s="14">
         <f t="shared" ref="J3:J5" si="0">SUM(G3:I3)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3" s="14"/>
       <c r="L3" s="55" t="s">
         <v>138</v>
       </c>
       <c r="M3" s="52">
-        <f>(G3+H4+I5)/COUNTA($C$2:$C$101)</f>
-        <v>0.83018867924528306</v>
+        <f>(G3+H4+I5)/COUNTA($C$2:$C$103)</f>
+        <v>0.83636363636363631</v>
       </c>
       <c r="N3" s="54" t="s">
         <v>139</v>
@@ -19526,12 +19540,12 @@
     </row>
     <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="5" t="str">
-        <f>'Human Grading'!A5</f>
-        <v>Composite State</v>
+        <f>'Human Grading'!A4</f>
+        <v>Transition</v>
       </c>
       <c r="B4" s="5" t="str">
-        <f>'Human Grading'!B5</f>
-        <v>On</v>
+        <f>'Human Grading'!B4</f>
+        <v>on (Off ⇒ On)</v>
       </c>
       <c r="C4" s="5">
         <f>'Human Grading'!C4</f>
@@ -19546,15 +19560,15 @@
         <v>0.5</v>
       </c>
       <c r="G4" s="56">
-        <f t="shared" ref="G4:I4" si="1">COUNTIFS($C$2:$C$47, $F4, $D$2:$D$47, G$2)</f>
+        <f>COUNTIFS($C$2:$C$49, $F4, $D$2:$D$49, G$2)</f>
         <v>6</v>
       </c>
       <c r="H4" s="14">
-        <f t="shared" si="1"/>
+        <f>COUNTIFS($C$2:$C$49, $F4, $D$2:$D$49, H$2)</f>
         <v>1</v>
       </c>
       <c r="I4" s="57">
-        <f t="shared" si="1"/>
+        <f>COUNTIFS($C$2:$C$49, $F4, $D$2:$D$49, I$2)</f>
         <v>0</v>
       </c>
       <c r="J4" s="14">
@@ -19566,8 +19580,8 @@
         <v>140</v>
       </c>
       <c r="M4" s="56">
-        <f t="array" ref="M4">SUMPRODUCT(J3:J5/COUNTA($C$2:$C$101), TRANSPOSE(G6:I6)/COUNTA($C$2:$C$101))</f>
-        <v>0.47098611605553575</v>
+        <f t="array" ref="M4">SUMPRODUCT(J3:J5/COUNTA($C$2:$C$103), TRANSPOSE(G6:I6)/COUNTA($C$2:$C$103))</f>
+        <v>0.46049586776859502</v>
       </c>
       <c r="N4" s="57" t="s">
         <v>141</v>
@@ -19575,12 +19589,12 @@
     </row>
     <row r="5" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="5" t="str">
-        <f>'Human Grading'!A2</f>
-        <v>State</v>
+        <f>'Human Grading'!A5</f>
+        <v>Composite State</v>
       </c>
       <c r="B5" s="5" t="str">
-        <f>'Human Grading'!B2</f>
-        <v>Initial state (→ Off)</v>
+        <f>'Human Grading'!B5</f>
+        <v>On</v>
       </c>
       <c r="C5" s="5">
         <f>'Human Grading'!C5</f>
@@ -19595,15 +19609,15 @@
         <v>1</v>
       </c>
       <c r="G5" s="58">
-        <f>COUNTIFS($C$2:$C$47, $F5, $D$2:$D$47, G$2)+MAX(C48-D48,0)+MAX(C49-D49,0)+MAX(C50-D50,0)+MAX(C51-D51,0)+MAX(C52-D52,0)+MAX(C53-D53,0)+MAX(C54-D54,0)</f>
+        <f>COUNTIFS($C$2:$C$49, $F5, $D$2:$D$49, G$2)+MAX(C50-D50,0)+MAX(C51-D51,0)+MAX(C52-D52,0)+MAX(C53-D53,0)+MAX(C54-D54,0)+MAX(C55-D55,0)+MAX(C56-D56,0)</f>
         <v>2</v>
       </c>
       <c r="H5" s="59">
-        <f>COUNTIFS($C$2:$C$47, $F5, $D$2:$D$47, H$2)</f>
+        <f>COUNTIFS($C$2:$C$49, $F5, $D$2:$D$49, H$2)</f>
         <v>0</v>
       </c>
       <c r="I5" s="60">
-        <f>COUNTIFS($C$2:$C$47, $F5, $D$2:$D$47, I$2)+ SUM(MIN(C48,D48), MIN(C49,D49), MIN(C50,D50), MIN(C51,D51), MIN(C52,D52), MIN(C53,D53), MIN(C54,D54))</f>
+        <f>COUNTIFS($C$2:$C$49, $F5, $D$2:$D$49, I$2)+ SUM(MIN(C50,D50), MIN(C51,D51), MIN(C52,D52), MIN(C53,D53), MIN(C54,D54), MIN(C55,D55), MIN(C56,D56))</f>
         <v>31</v>
       </c>
       <c r="J5" s="14">
@@ -19616,7 +19630,7 @@
       </c>
       <c r="M5" s="58">
         <f>(M3-M4)/(1-M4)</f>
-        <v>0.67900403768506068</v>
+        <v>0.6966911764705882</v>
       </c>
       <c r="N5" s="60" t="s">
         <v>142</v>
@@ -19624,12 +19638,12 @@
     </row>
     <row r="6" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="5" t="str">
-        <f>'Human Grading'!A7</f>
-        <v>Composite State</v>
+        <f>'Human Grading'!A6</f>
+        <v>Transition</v>
       </c>
       <c r="B6" s="5" t="str">
-        <f>'Human Grading'!B7</f>
-        <v>Setup</v>
+        <f>'Human Grading'!B6</f>
+        <v>on =&gt; off</v>
       </c>
       <c r="C6" s="5">
         <f>'Human Grading'!C6</f>
@@ -19644,15 +19658,15 @@
         <v>143</v>
       </c>
       <c r="G6" s="14">
-        <f t="shared" ref="G6:I6" si="2">SUM(G3:G5)</f>
-        <v>20</v>
+        <f t="shared" ref="G6:I6" si="1">SUM(G3:G5)</f>
+        <v>22</v>
       </c>
       <c r="H6" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I6" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="J6" s="14"/>
@@ -19661,12 +19675,12 @@
     </row>
     <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="5" t="str">
-        <f>'Human Grading'!A8</f>
-        <v>State</v>
+        <f>'Human Grading'!A7</f>
+        <v>Composite State</v>
       </c>
       <c r="B7" s="5" t="str">
-        <f>'Human Grading'!B8</f>
-        <v>Initial state (Setup → Medium)</v>
+        <f>'Human Grading'!B7</f>
+        <v>Setup</v>
       </c>
       <c r="C7" s="5">
         <f>'Human Grading'!C7</f>
@@ -19683,42 +19697,42 @@
     </row>
     <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="5" t="str">
+        <f>'Human Grading'!A8</f>
+        <v>State</v>
+      </c>
+      <c r="B8" s="5" t="str">
+        <f>'Human Grading'!B8</f>
+        <v>Initial state (Setup → Medium)</v>
+      </c>
+      <c r="C8" s="5">
+        <f>'Human Grading'!C8</f>
+        <v>1</v>
+      </c>
+      <c r="D8" s="5">
+        <f>'LLM Grading'!C8</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="44"/>
+      <c r="F8" s="68" t="s">
+        <v>144</v>
+      </c>
+      <c r="G8" s="69"/>
+      <c r="H8" s="69"/>
+      <c r="I8" s="69"/>
+      <c r="L8" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="M8" s="73"/>
+      <c r="N8" s="73"/>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="5" t="str">
         <f>'Human Grading'!A9</f>
         <v>Action</v>
       </c>
-      <c r="B8" s="5" t="str">
+      <c r="B9" s="5" t="str">
         <f>'Human Grading'!B9</f>
         <v>delay=0; selectFirstCourse()</v>
-      </c>
-      <c r="C8" s="5">
-        <f>'Human Grading'!C8</f>
-        <v>1</v>
-      </c>
-      <c r="D8" s="5">
-        <f>'LLM Grading'!C8</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="44"/>
-      <c r="F8" s="69" t="s">
-        <v>144</v>
-      </c>
-      <c r="G8" s="70"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="70"/>
-      <c r="L8" s="71" t="s">
-        <v>145</v>
-      </c>
-      <c r="M8" s="72"/>
-      <c r="N8" s="72"/>
-    </row>
-    <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="5" t="str">
-        <f>'Human Grading'!A10</f>
-        <v>State</v>
-      </c>
-      <c r="B9" s="5" t="str">
-        <f>'Human Grading'!B10</f>
-        <v>Medium</v>
       </c>
       <c r="C9" s="5">
         <f>'Human Grading'!C9</f>
@@ -19757,12 +19771,12 @@
     </row>
     <row r="10" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="5" t="str">
-        <f>'Human Grading'!A11</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A10</f>
+        <v>State</v>
       </c>
       <c r="B10" s="5" t="str">
-        <f>'Human Grading'!B11</f>
-        <v>setup initial state =&gt; medium</v>
+        <f>'Human Grading'!B10</f>
+        <v>Medium</v>
       </c>
       <c r="C10" s="5">
         <f>'Human Grading'!C10</f>
@@ -19777,27 +19791,27 @@
         <v>0</v>
       </c>
       <c r="G10" s="52">
-        <f t="shared" ref="G10:H10" si="3">COUNTIFS($A$2:$A$91,$F$9,$C$2:$C$91,$F10,$D$2:$D$91,G$9)</f>
-        <v>0</v>
+        <f>COUNTIFS($A$2:$A$93,$F$9,$C$2:$C$93,$F10,$D$2:$D$93,G$9)</f>
+        <v>1</v>
       </c>
       <c r="H10" s="53">
-        <f t="shared" si="3"/>
+        <f>COUNTIFS($A$2:$A$93,$F$9,$C$2:$C$93,$F10,$D$2:$D$93,H$9)</f>
         <v>0</v>
       </c>
       <c r="I10" s="54">
-        <f>COUNTIFS($A$2:$A$47,$F$9,$C$2:$C$47,$F10,$D$2:$D$47,I$9)+MAX(D48-C48,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$9,$C$2:$C$49,$F10,$D$2:$D$49,I$9)+MAX(D50-C50,0)</f>
         <v>0</v>
       </c>
       <c r="J10" s="14">
-        <f t="shared" ref="J10:J12" si="4">SUM(G10:I10)</f>
-        <v>0</v>
+        <f t="shared" ref="J10:J12" si="2">SUM(G10:I10)</f>
+        <v>1</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="55" t="s">
         <v>138</v>
       </c>
       <c r="M10" s="52">
-        <f>(G10+H11+I12)/COUNTIF($A$2:$A$101,F9)</f>
+        <f>(G10+H11+I12)/COUNTIF($A$2:$A$103,F9)</f>
         <v>0.69230769230769229</v>
       </c>
       <c r="N10" s="54" t="s">
@@ -19806,12 +19820,12 @@
     </row>
     <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="5" t="str">
-        <f>'Human Grading'!A12</f>
+        <f>'Human Grading'!A11</f>
         <v>Transition</v>
       </c>
       <c r="B11" s="5" t="str">
-        <f>'Human Grading'!B12</f>
-        <v>medium =&gt; dark</v>
+        <f>'Human Grading'!B11</f>
+        <v>setup initial state =&gt; medium</v>
       </c>
       <c r="C11" s="5">
         <f>'Human Grading'!C11</f>
@@ -19826,19 +19840,19 @@
         <v>0.5</v>
       </c>
       <c r="G11" s="56">
-        <f t="shared" ref="G11:I11" si="5">COUNTIFS($A$2:$A$91,$F$9,$C$2:$C$91,$F11,$D$2:$D$91,G$9)</f>
-        <v>2</v>
+        <f>COUNTIFS($A$2:$A$93,$F$9,$C$2:$C$93,$F11,$D$2:$D$93,G$9)</f>
+        <v>3</v>
       </c>
       <c r="H11" s="14">
-        <f t="shared" si="5"/>
-        <v>1</v>
+        <f>COUNTIFS($A$2:$A$93,$F$9,$C$2:$C$93,$F11,$D$2:$D$93,H$9)</f>
+        <v>0</v>
       </c>
       <c r="I11" s="57">
-        <f t="shared" si="5"/>
+        <f>COUNTIFS($A$2:$A$93,$F$9,$C$2:$C$93,$F11,$D$2:$D$93,I$9)</f>
         <v>0</v>
       </c>
       <c r="J11" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="K11" s="14"/>
@@ -19846,8 +19860,8 @@
         <v>140</v>
       </c>
       <c r="M11" s="56">
-        <f t="array" ref="M11">SUMPRODUCT(J10:J12/COUNTIF($A$2:$A$101,F9), TRANSPOSE(G13:I13)/COUNTIF($A$2:$A$101,F9))</f>
-        <v>0.4437869822485207</v>
+        <f t="array" ref="M11">SUMPRODUCT(J10:J12/COUNTIF($A$2:$A$103,F9), TRANSPOSE(G13:I13)/COUNTIF($A$2:$A$103,F9))</f>
+        <v>0.45562130177514792</v>
       </c>
       <c r="N11" s="57" t="s">
         <v>141</v>
@@ -19855,12 +19869,12 @@
     </row>
     <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="5" t="str">
-        <f>'Human Grading'!A13</f>
-        <v>State</v>
+        <f>'Human Grading'!A12</f>
+        <v>Transition</v>
       </c>
       <c r="B12" s="5" t="str">
-        <f>'Human Grading'!B13</f>
-        <v>Dark</v>
+        <f>'Human Grading'!B12</f>
+        <v>medium =&gt; dark</v>
       </c>
       <c r="C12" s="5">
         <f>'Human Grading'!C12</f>
@@ -19875,19 +19889,19 @@
         <v>1</v>
       </c>
       <c r="G12" s="58">
-        <f>COUNTIFS($A$2:$A$47,$F$9,$C$2:$C$47,$F12,$D$2:$D$47,G$9)+MAX(C48-D48,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$9,$C$2:$C$49,$F12,$D$2:$D$49,G$9)+MAX(C50-D50,0)</f>
         <v>1</v>
       </c>
       <c r="H12" s="59">
-        <f>COUNTIFS($A$2:$A$91,$F$9,$C$2:$C$91,$F12,$D$2:$D$91,H$9)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$9,$C$2:$C$93,$F12,$D$2:$D$93,H$9)</f>
         <v>0</v>
       </c>
       <c r="I12" s="60">
-        <f>COUNTIFS($A$2:$A$47,$F$9,$C$2:$C$47,$F12,$D$2:$D$47,I$9)+MIN(C48-D48)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$9,$C$2:$C$49,$F12,$D$2:$D$49,I$9)+MIN(C50-D50)</f>
         <v>8</v>
       </c>
       <c r="J12" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="K12" s="14"/>
@@ -19896,7 +19910,7 @@
       </c>
       <c r="M12" s="58">
         <f>(M10-M11)/(1-M11)</f>
-        <v>0.44680851063829791</v>
+        <v>0.43478260869565216</v>
       </c>
       <c r="N12" s="60" t="s">
         <v>142</v>
@@ -19904,12 +19918,12 @@
     </row>
     <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="5" t="str">
-        <f>'Human Grading'!A14</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A13</f>
+        <v>State</v>
       </c>
       <c r="B13" s="5" t="str">
-        <f>'Human Grading'!B14</f>
-        <v>dark =&gt; light</v>
+        <f>'Human Grading'!B13</f>
+        <v>Dark</v>
       </c>
       <c r="C13" s="5">
         <f>'Human Grading'!C13</f>
@@ -19924,15 +19938,15 @@
         <v>143</v>
       </c>
       <c r="G13" s="14">
-        <f t="shared" ref="G13:I13" si="6">SUM(G10:G12)</f>
-        <v>3</v>
+        <f t="shared" ref="G13:I13" si="3">SUM(G10:G12)</f>
+        <v>5</v>
       </c>
       <c r="H13" s="14">
-        <f t="shared" si="6"/>
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="I13" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>8</v>
       </c>
       <c r="J13" s="14"/>
@@ -19941,12 +19955,12 @@
     </row>
     <row r="14" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="5" t="str">
-        <f>'Human Grading'!A15</f>
-        <v>State</v>
+        <f>'Human Grading'!A14</f>
+        <v>Transition</v>
       </c>
       <c r="B14" s="5" t="str">
-        <f>'Human Grading'!B15</f>
-        <v>Light</v>
+        <f>'Human Grading'!B14</f>
+        <v>dark =&gt; light</v>
       </c>
       <c r="C14" s="5">
         <f>'Human Grading'!C14</f>
@@ -19960,12 +19974,12 @@
     </row>
     <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="5" t="str">
-        <f>'Human Grading'!A16</f>
-        <v>History State</v>
+        <f>'Human Grading'!A15</f>
+        <v>State</v>
       </c>
       <c r="B15" s="5" t="str">
-        <f>'Human Grading'!B16</f>
-        <v>H</v>
+        <f>'Human Grading'!B15</f>
+        <v>Light</v>
       </c>
       <c r="C15" s="5">
         <f>'Human Grading'!C15</f>
@@ -19976,26 +19990,26 @@
         <v>0</v>
       </c>
       <c r="E15" s="44"/>
-      <c r="F15" s="69" t="s">
+      <c r="F15" s="68" t="s">
         <v>146</v>
       </c>
-      <c r="G15" s="70"/>
-      <c r="H15" s="70"/>
-      <c r="I15" s="70"/>
-      <c r="L15" s="71" t="s">
+      <c r="G15" s="69"/>
+      <c r="H15" s="69"/>
+      <c r="I15" s="69"/>
+      <c r="L15" s="72" t="s">
         <v>147</v>
       </c>
-      <c r="M15" s="72"/>
-      <c r="N15" s="72"/>
+      <c r="M15" s="73"/>
+      <c r="N15" s="73"/>
     </row>
     <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="5" t="str">
-        <f>'Human Grading'!A17</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A16</f>
+        <v>History State</v>
       </c>
       <c r="B16" s="5" t="str">
-        <f>'Human Grading'!B17</f>
-        <v>setup =&gt; H</v>
+        <f>'Human Grading'!B16</f>
+        <v>H</v>
       </c>
       <c r="C16" s="5">
         <f>'Human Grading'!C16</f>
@@ -20034,12 +20048,12 @@
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="5" t="str">
-        <f>'Human Grading'!A18</f>
-        <v>Action</v>
+        <f>'Human Grading'!A17</f>
+        <v>Transition</v>
       </c>
       <c r="B17" s="5" t="str">
-        <f>'Human Grading'!B18</f>
-        <v>selectNextCourse()</v>
+        <f>'Human Grading'!B17</f>
+        <v>setup =&gt; H</v>
       </c>
       <c r="C17" s="5">
         <f>'Human Grading'!C17</f>
@@ -20054,28 +20068,28 @@
         <v>0</v>
       </c>
       <c r="G17" s="52">
-        <f t="shared" ref="G17:H17" si="7">COUNTIFS($A$2:$A$91,$F$16,$C$2:$C$91,$F17,$D$2:$D$91,G$16)</f>
-        <v>5</v>
+        <f>COUNTIFS($A$2:$A$93,$F$16,$C$2:$C$93,$F17,$D$2:$D$93,G$16)</f>
+        <v>2</v>
       </c>
       <c r="H17" s="53">
-        <f t="shared" si="7"/>
+        <f>COUNTIFS($A$2:$A$93,$F$16,$C$2:$C$93,$F17,$D$2:$D$93,H$16)</f>
         <v>0</v>
       </c>
       <c r="I17" s="54">
-        <f>COUNTIFS($A$2:$A$47,$F$16,$C$2:$C$47,$F17,$D$2:$D$47,I$16) + MAX(D49-C49,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$16,$C$2:$C$49,$F17,$D$2:$D$49,I$16) + MAX(D51-C51,0)</f>
         <v>0</v>
       </c>
       <c r="J17" s="14">
-        <f t="shared" ref="J17:J19" si="8">SUM(G17:I17)</f>
-        <v>5</v>
+        <f t="shared" ref="J17:J19" si="4">SUM(G17:I17)</f>
+        <v>2</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="55" t="s">
         <v>138</v>
       </c>
       <c r="M17" s="52">
-        <f>(G17+H18+I19)/COUNTIF($A$2:$A$101,F16)</f>
-        <v>0.82352941176470584</v>
+        <f>(G17+H18+I19)/COUNTIF($A$2:$A$103,F16)</f>
+        <v>0.84210526315789469</v>
       </c>
       <c r="N17" s="54" t="s">
         <v>139</v>
@@ -20083,12 +20097,12 @@
     </row>
     <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="5" t="str">
-        <f>'Human Grading'!A19</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A18</f>
+        <v>Action</v>
       </c>
       <c r="B18" s="5" t="str">
-        <f>'Human Grading'!B19</f>
-        <v>plus (Setup ⇒ Setup)</v>
+        <f>'Human Grading'!B18</f>
+        <v>selectNextCourse()</v>
       </c>
       <c r="C18" s="5">
         <f>'Human Grading'!C18</f>
@@ -20103,19 +20117,19 @@
         <v>0.5</v>
       </c>
       <c r="G18" s="56">
-        <f t="shared" ref="G18:I18" si="9">COUNTIFS($A$2:$A$91,$F$16,$C$2:$C$91,$F18,$D$2:$D$91,G$16)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$16,$C$2:$C$93,$F18,$D$2:$D$93,G$16)</f>
         <v>3</v>
       </c>
       <c r="H18" s="14">
-        <f t="shared" si="9"/>
+        <f>COUNTIFS($A$2:$A$93,$F$16,$C$2:$C$93,$F18,$D$2:$D$93,H$16)</f>
         <v>0</v>
       </c>
       <c r="I18" s="57">
-        <f t="shared" si="9"/>
+        <f>COUNTIFS($A$2:$A$93,$F$16,$C$2:$C$93,$F18,$D$2:$D$93,I$16)</f>
         <v>0</v>
       </c>
       <c r="J18" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="K18" s="14"/>
@@ -20123,8 +20137,8 @@
         <v>140</v>
       </c>
       <c r="M18" s="56">
-        <f t="array" ref="M18">SUMPRODUCT(J17:J19/COUNTIF($A$2:$A$101,F16), TRANSPOSE(G20:I20)/COUNTIF($A$2:$A$101,F16))</f>
-        <v>0.41868512110726647</v>
+        <f t="array" ref="M18">SUMPRODUCT(J17:J19/COUNTIF($A$2:$A$103,F16), TRANSPOSE(G20:I20)/COUNTIF($A$2:$A$103,F16))</f>
+        <v>0.57063711911357329</v>
       </c>
       <c r="N18" s="57" t="s">
         <v>141</v>
@@ -20132,12 +20146,12 @@
     </row>
     <row r="19" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="5" t="str">
-        <f>'Human Grading'!A20</f>
-        <v>Guard</v>
+        <f>'Human Grading'!A19</f>
+        <v>Transition</v>
       </c>
       <c r="B19" s="5" t="str">
-        <f>'Human Grading'!B20</f>
-        <v>[delay &lt;= 17*60+50]</v>
+        <f>'Human Grading'!B19</f>
+        <v>plus (Setup ⇒ Setup)</v>
       </c>
       <c r="C19" s="5">
         <f>'Human Grading'!C19</f>
@@ -20152,20 +20166,20 @@
         <v>1</v>
       </c>
       <c r="G19" s="58">
-        <f>COUNTIFS($A$2:$A$47,$F$16,$C$2:$C$47,$F19,$D$2:$D$47,G$16)+MAX(C49-D49,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$16,$C$2:$C$49,$F19,$D$2:$D$49,G$16)+MAX(C51-D51,0)</f>
         <v>0</v>
       </c>
       <c r="H19" s="59">
-        <f>COUNTIFS($A$2:$A$91,$F$16,$C$2:$C$91,$F19,$D$2:$D$91,H$16)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$16,$C$2:$C$93,$F19,$D$2:$D$93,H$16)</f>
         <v>0</v>
       </c>
       <c r="I19" s="60">
-        <f>COUNTIFS($A$2:$A$47,$F$16,$C$2:$C$47,$F19,$D$2:$D$47,I$16) + MIN(C49,D49)</f>
-        <v>9</v>
+        <f>COUNTIFS($A$2:$A$49,$F$16,$C$2:$C$49,$F19,$D$2:$D$49,I$16) + MIN(C51,D51)</f>
+        <v>14</v>
       </c>
       <c r="J19" s="14">
-        <f t="shared" si="8"/>
-        <v>9</v>
+        <f t="shared" si="4"/>
+        <v>14</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="55" t="s">
@@ -20173,7 +20187,7 @@
       </c>
       <c r="M19" s="58">
         <f>(M17-M18)/(1-M18)</f>
-        <v>0.69642857142857129</v>
+        <v>0.63225806451612898</v>
       </c>
       <c r="N19" s="60" t="s">
         <v>142</v>
@@ -20181,12 +20195,12 @@
     </row>
     <row r="20" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="5" t="str">
-        <f>'Human Grading'!A21</f>
-        <v>Action</v>
+        <f>'Human Grading'!A20</f>
+        <v>Guard</v>
       </c>
       <c r="B20" s="5" t="str">
-        <f>'Human Grading'!B21</f>
-        <v>delay = delay + 10</v>
+        <f>'Human Grading'!B20</f>
+        <v>[delay &lt;= 17*60+50]</v>
       </c>
       <c r="C20" s="5">
         <f>'Human Grading'!C20</f>
@@ -20201,16 +20215,16 @@
         <v>143</v>
       </c>
       <c r="G20" s="14">
-        <f t="shared" ref="G20:I20" si="10">SUM(G17:G19)</f>
-        <v>8</v>
+        <f t="shared" ref="G20:I20" si="5">SUM(G17:G19)</f>
+        <v>5</v>
       </c>
       <c r="H20" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="I20" s="14">
-        <f t="shared" si="10"/>
-        <v>9</v>
+        <f t="shared" si="5"/>
+        <v>14</v>
       </c>
       <c r="J20" s="14"/>
       <c r="L20" s="14"/>
@@ -20218,61 +20232,61 @@
     </row>
     <row r="21" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="5" t="str">
+        <f>'Human Grading'!A21</f>
+        <v>Action</v>
+      </c>
+      <c r="B21" s="5" t="str">
+        <f>'Human Grading'!B21</f>
+        <v>delay = delay + 10</v>
+      </c>
+      <c r="C21" s="5">
+        <f>'Human Grading'!C21</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="5">
+        <f>'LLM Grading'!C21</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="44"/>
+    </row>
+    <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="5" t="str">
         <f>'Human Grading'!A22</f>
         <v>Transition</v>
       </c>
-      <c r="B21" s="5" t="str">
+      <c r="B22" s="5" t="str">
         <f>'Human Grading'!B22</f>
         <v>minus (Setup ⇒ Setup)</v>
       </c>
-      <c r="C21" s="5">
-        <f>'Human Grading'!C21</f>
-        <v>0</v>
-      </c>
-      <c r="D21" s="5">
-        <f>'LLM Grading'!C21</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="44"/>
-    </row>
-    <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="5" t="str">
+      <c r="C22" s="5">
+        <f>'Human Grading'!C22</f>
+        <v>1</v>
+      </c>
+      <c r="D22" s="5">
+        <f>'LLM Grading'!C22</f>
+        <v>1</v>
+      </c>
+      <c r="E22" s="44"/>
+      <c r="F22" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="G22" s="69"/>
+      <c r="H22" s="69"/>
+      <c r="I22" s="69"/>
+      <c r="L22" s="72" t="s">
+        <v>149</v>
+      </c>
+      <c r="M22" s="73"/>
+      <c r="N22" s="73"/>
+    </row>
+    <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="5" t="str">
         <f>'Human Grading'!A23</f>
         <v>Guard</v>
       </c>
-      <c r="B22" s="5" t="str">
+      <c r="B23" s="5" t="str">
         <f>'Human Grading'!B23</f>
         <v>[delay &gt;= 10]</v>
-      </c>
-      <c r="C22" s="5">
-        <f>'Human Grading'!C22</f>
-        <v>1</v>
-      </c>
-      <c r="D22" s="5">
-        <f>'LLM Grading'!C22</f>
-        <v>1</v>
-      </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="69" t="s">
-        <v>148</v>
-      </c>
-      <c r="G22" s="70"/>
-      <c r="H22" s="70"/>
-      <c r="I22" s="70"/>
-      <c r="L22" s="71" t="s">
-        <v>149</v>
-      </c>
-      <c r="M22" s="72"/>
-      <c r="N22" s="72"/>
-    </row>
-    <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="5" t="str">
-        <f>'Human Grading'!A24</f>
-        <v>Action</v>
-      </c>
-      <c r="B23" s="5" t="str">
-        <f>'Human Grading'!B24</f>
-        <v>delay = delay - 10</v>
       </c>
       <c r="C23" s="5">
         <f>'Human Grading'!C23</f>
@@ -20311,12 +20325,12 @@
     </row>
     <row r="24" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="str">
-        <f>'Human Grading'!A25</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A24</f>
+        <v>Action</v>
       </c>
       <c r="B24" s="5" t="str">
-        <f>'Human Grading'!B25</f>
-        <v>start (Setup ⇒ Countdown)</v>
+        <f>'Human Grading'!B24</f>
+        <v>delay = delay - 10</v>
       </c>
       <c r="C24" s="5">
         <f>'Human Grading'!C24</f>
@@ -20331,27 +20345,27 @@
         <v>0</v>
       </c>
       <c r="G24" s="52">
-        <f t="shared" ref="G24:H24" si="11">COUNTIFS($A$2:$A$91,$F$23,$C$2:$C$91,$F24,$D$2:$D$91,G$23)</f>
-        <v>2</v>
+        <f>COUNTIFS($A$2:$A$93,$F$23,$C$2:$C$93,$F24,$D$2:$D$93,G$23)</f>
+        <v>1</v>
       </c>
       <c r="H24" s="53">
-        <f t="shared" si="11"/>
+        <f>COUNTIFS($A$2:$A$93,$F$23,$C$2:$C$93,$F24,$D$2:$D$93,H$23)</f>
         <v>0</v>
       </c>
       <c r="I24" s="54">
-        <f>COUNTIFS($A$2:$A$47,$F$23,$C$2:$C$47,$F24,$D$2:$D$47,I$23) + MAX(D52-C52,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$23,$C$2:$C$49,$F24,$D$2:$D$49,I$23) + MAX(D54-C54,0)</f>
         <v>0</v>
       </c>
       <c r="J24" s="14">
-        <f t="shared" ref="J24:J26" si="12">SUM(G24:I24)</f>
-        <v>2</v>
+        <f t="shared" ref="J24:J26" si="6">SUM(G24:I24)</f>
+        <v>1</v>
       </c>
       <c r="K24" s="14"/>
       <c r="L24" s="55" t="s">
         <v>138</v>
       </c>
       <c r="M24" s="52">
-        <f>(G24+H25+I26)/COUNTIF($A$2:$A$101,F23)</f>
+        <f>(G24+H25+I26)/COUNTIF($A$2:$A$103,F23)</f>
         <v>1</v>
       </c>
       <c r="N24" s="54" t="s">
@@ -20360,12 +20374,12 @@
     </row>
     <row r="25" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="str">
-        <f>'Human Grading'!A26</f>
-        <v>Guard</v>
+        <f>'Human Grading'!A25</f>
+        <v>Transition</v>
       </c>
       <c r="B25" s="5" t="str">
-        <f>'Human Grading'!B26</f>
-        <v>[delay &gt; 0]</v>
+        <f>'Human Grading'!B25</f>
+        <v>start (Setup ⇒ Countdown)</v>
       </c>
       <c r="C25" s="5">
         <f>'Human Grading'!C25</f>
@@ -20380,41 +20394,41 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="56">
-        <f t="shared" ref="G25:I25" si="13">COUNTIFS($A$2:$A$91,$F$23,$C$2:$C$91,$F25,$D$2:$D$91,G$23)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$23,$C$2:$C$93,$F25,$D$2:$D$93,G$23)</f>
         <v>0</v>
       </c>
       <c r="H25" s="14">
-        <f t="shared" si="13"/>
-        <v>0</v>
+        <f>COUNTIFS($A$2:$A$93,$F$23,$C$2:$C$93,$F25,$D$2:$D$93,H$23)</f>
+        <v>1</v>
       </c>
       <c r="I25" s="57">
-        <f t="shared" si="13"/>
+        <f>COUNTIFS($A$2:$A$93,$F$23,$C$2:$C$93,$F25,$D$2:$D$93,I$23)</f>
         <v>0</v>
       </c>
       <c r="J25" s="14">
-        <f t="shared" si="12"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>1</v>
       </c>
       <c r="K25" s="14"/>
       <c r="L25" s="55" t="s">
         <v>140</v>
       </c>
       <c r="M25" s="56">
-        <f t="array" ref="M25">SUMPRODUCT(J24:J26/COUNTIF($A$2:$A$101,F23), TRANSPOSE(G27:I27)/COUNTIF($A$2:$A$101,F23))</f>
-        <v>0.5</v>
+        <f t="array" ref="M25">SUMPRODUCT(J24:J26/COUNTIF($A$2:$A$103,F23), TRANSPOSE(G27:I27)/COUNTIF($A$2:$A$103,F23))</f>
+        <v>0.375</v>
       </c>
       <c r="N25" s="57" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="str">
-        <f>'Human Grading'!A27</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A26</f>
+        <v>Guard</v>
       </c>
       <c r="B26" s="5" t="str">
-        <f>'Human Grading'!B27</f>
-        <v>start (Setup ⇒ Baking)</v>
+        <f>'Human Grading'!B26</f>
+        <v>[delay &gt; 0]</v>
       </c>
       <c r="C26" s="5">
         <f>'Human Grading'!C26</f>
@@ -20429,19 +20443,19 @@
         <v>1</v>
       </c>
       <c r="G26" s="58">
-        <f>COUNTIFS($A$2:$A$47,$F$23,$C$2:$C$47,$F26,$D$2:$D$47,G$23) + MAX(C52-D52,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$23,$C$2:$C$49,$F26,$D$2:$D$49,G$23) + MAX(C54-D54,0)</f>
         <v>0</v>
       </c>
       <c r="H26" s="59">
-        <f>COUNTIFS($A$2:$A$91,$F$23,$C$2:$C$91,$F26,$D$2:$D$91,H$23)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$23,$C$2:$C$93,$F26,$D$2:$D$93,H$23)</f>
         <v>0</v>
       </c>
       <c r="I26" s="60">
-        <f>COUNTIFS($A$2:$A$47,$F$23,$C$2:$C$47,$F26,$D$2:$D$47,I$23) + MIN(C52,D52)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$23,$C$2:$C$49,$F26,$D$2:$D$49,I$23) + MIN(C54,D54)</f>
         <v>2</v>
       </c>
       <c r="J26" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="K26" s="14"/>
@@ -20458,12 +20472,12 @@
     </row>
     <row r="27" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="str">
-        <f>'Human Grading'!A28</f>
-        <v>Guard</v>
+        <f>'Human Grading'!A27</f>
+        <v>Transition</v>
       </c>
       <c r="B27" s="5" t="str">
-        <f>'Human Grading'!B28</f>
-        <v>[delay == 0]</v>
+        <f>'Human Grading'!B27</f>
+        <v>start (Setup ⇒ Baking)</v>
       </c>
       <c r="C27" s="5">
         <f>'Human Grading'!C27</f>
@@ -20478,15 +20492,15 @@
         <v>143</v>
       </c>
       <c r="G27" s="14">
-        <f t="shared" ref="G27:I27" si="14">SUM(G24:G26)</f>
-        <v>2</v>
+        <f t="shared" ref="G27:I27" si="7">SUM(G24:G26)</f>
+        <v>1</v>
       </c>
       <c r="H27" s="14">
-        <f t="shared" si="14"/>
-        <v>0</v>
+        <f t="shared" si="7"/>
+        <v>1</v>
       </c>
       <c r="I27" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="J27" s="14"/>
@@ -20495,61 +20509,61 @@
     </row>
     <row r="28" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="5" t="str">
+        <f>'Human Grading'!A28</f>
+        <v>Guard</v>
+      </c>
+      <c r="B28" s="5" t="str">
+        <f>'Human Grading'!B28</f>
+        <v>[delay == 0]</v>
+      </c>
+      <c r="C28" s="5">
+        <f>'Human Grading'!C28</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="5">
+        <f>'LLM Grading'!C28</f>
+        <v>1</v>
+      </c>
+      <c r="E28" s="44"/>
+    </row>
+    <row r="29" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="str">
         <f>'Human Grading'!A29</f>
         <v>State</v>
       </c>
-      <c r="B28" s="5" t="str">
+      <c r="B29" s="5" t="str">
         <f>'Human Grading'!B29</f>
         <v>Countdown</v>
       </c>
-      <c r="C28" s="5">
-        <f>'Human Grading'!C28</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="5">
-        <f>'LLM Grading'!C28</f>
-        <v>1</v>
-      </c>
-      <c r="E28" s="44"/>
-    </row>
-    <row r="29" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="5" t="str">
+      <c r="C29" s="5">
+        <f>'Human Grading'!C29</f>
+        <v>1</v>
+      </c>
+      <c r="D29" s="5">
+        <f>'LLM Grading'!C29</f>
+        <v>1</v>
+      </c>
+      <c r="E29" s="44"/>
+      <c r="F29" s="68" t="s">
+        <v>150</v>
+      </c>
+      <c r="G29" s="69"/>
+      <c r="H29" s="69"/>
+      <c r="I29" s="69"/>
+      <c r="L29" s="72" t="s">
+        <v>151</v>
+      </c>
+      <c r="M29" s="73"/>
+      <c r="N29" s="73"/>
+    </row>
+    <row r="30" spans="1:14" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="str">
         <f>'Human Grading'!A30</f>
         <v>Action</v>
       </c>
-      <c r="B29" s="5" t="str">
+      <c r="B30" s="5" t="str">
         <f>'Human Grading'!B30</f>
         <v>setCourseTimes()</v>
-      </c>
-      <c r="C29" s="5">
-        <f>'Human Grading'!C29</f>
-        <v>1</v>
-      </c>
-      <c r="D29" s="5">
-        <f>'LLM Grading'!C29</f>
-        <v>1</v>
-      </c>
-      <c r="E29" s="44"/>
-      <c r="F29" s="69" t="s">
-        <v>150</v>
-      </c>
-      <c r="G29" s="70"/>
-      <c r="H29" s="70"/>
-      <c r="I29" s="70"/>
-      <c r="L29" s="71" t="s">
-        <v>151</v>
-      </c>
-      <c r="M29" s="72"/>
-      <c r="N29" s="72"/>
-    </row>
-    <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="5" t="str">
-        <f>'Human Grading'!A31</f>
-        <v>Transition</v>
-      </c>
-      <c r="B30" s="5" t="str">
-        <f>'Human Grading'!B31</f>
-        <v>Countdown =&gt; baking</v>
       </c>
       <c r="C30" s="5">
         <f>'Human Grading'!C30</f>
@@ -20588,12 +20602,12 @@
     </row>
     <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="5" t="str">
-        <f>'Human Grading'!A32</f>
+        <f>'Human Grading'!A31</f>
         <v>Transition</v>
       </c>
       <c r="B31" s="5" t="str">
-        <f>'Human Grading'!B32</f>
-        <v>Countdown =&gt; setup</v>
+        <f>'Human Grading'!B31</f>
+        <v>Countdown =&gt; baking</v>
       </c>
       <c r="C31" s="5">
         <f>'Human Grading'!C31</f>
@@ -20608,28 +20622,28 @@
         <v>0</v>
       </c>
       <c r="G31" s="52">
-        <f t="shared" ref="G31:H31" si="15">COUNTIFS($A$2:$A$91,$F$30,$C$2:$C$91,$F31,$D$2:$D$91,G$30)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$30,$C$2:$C$93,$F31,$D$2:$D$93,G$30)</f>
         <v>1</v>
       </c>
       <c r="H31" s="53">
-        <f t="shared" si="15"/>
+        <f>COUNTIFS($A$2:$A$93,$F$30,$C$2:$C$93,$F31,$D$2:$D$93,H$30)</f>
         <v>0</v>
       </c>
       <c r="I31" s="54">
-        <f>COUNTIFS($A$2:$A$47,$F$30,$C$2:$C$47,$F31,$D$2:$D$47,I$30) + MAX(D50-C50,0)</f>
-        <v>0</v>
+        <f>COUNTIFS($A$2:$A$49,$F$30,$C$2:$C$49,$F31,$D$2:$D$49,I$30) + MAX(D52-C52,0)</f>
+        <v>1</v>
       </c>
       <c r="J31" s="14">
-        <f t="shared" ref="J31:J33" si="16">SUM(G31:I31)</f>
-        <v>1</v>
+        <f t="shared" ref="J31:J33" si="8">SUM(G31:I31)</f>
+        <v>2</v>
       </c>
       <c r="K31" s="14"/>
       <c r="L31" s="55" t="s">
         <v>138</v>
       </c>
       <c r="M31" s="52">
-        <f>(G31+H32+I33)/COUNTIF($A$2:$A$101,F30)</f>
-        <v>1</v>
+        <f>(G31+H32+I33)/COUNTIF($A$2:$A$103,F30)</f>
+        <v>0.8</v>
       </c>
       <c r="N31" s="54" t="s">
         <v>139</v>
@@ -20637,12 +20651,12 @@
     </row>
     <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="5" t="str">
-        <f>'Human Grading'!A33</f>
-        <v>Action</v>
+        <f>'Human Grading'!A32</f>
+        <v>Transition</v>
       </c>
       <c r="B32" s="5" t="str">
-        <f>'Human Grading'!B33</f>
-        <v>setCourseTimes()</v>
+        <f>'Human Grading'!B32</f>
+        <v>Countdown =&gt; setup</v>
       </c>
       <c r="C32" s="5">
         <f>'Human Grading'!C32</f>
@@ -20657,19 +20671,19 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="56">
-        <f t="shared" ref="G32:I32" si="17">COUNTIFS($A$2:$A$91,$F$30,$C$2:$C$91,$F32,$D$2:$D$91,G$30)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$30,$C$2:$C$93,$F32,$D$2:$D$93,G$30)</f>
         <v>0</v>
       </c>
       <c r="H32" s="14">
-        <f t="shared" si="17"/>
+        <f>COUNTIFS($A$2:$A$93,$F$30,$C$2:$C$93,$F32,$D$2:$D$93,H$30)</f>
         <v>0</v>
       </c>
       <c r="I32" s="57">
-        <f t="shared" si="17"/>
+        <f>COUNTIFS($A$2:$A$93,$F$30,$C$2:$C$93,$F32,$D$2:$D$93,I$30)</f>
         <v>0</v>
       </c>
       <c r="J32" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="K32" s="14"/>
@@ -20677,21 +20691,21 @@
         <v>140</v>
       </c>
       <c r="M32" s="56">
-        <f t="array" ref="M32">SUMPRODUCT(J31:J33/COUNTIF($A$2:$A$101,F30), TRANSPOSE(G34:I34)/COUNTIF($A$2:$A$101,F30))</f>
-        <v>0.68000000000000016</v>
+        <f t="array" ref="M32">SUMPRODUCT(J31:J33/COUNTIF($A$2:$A$103,F30), TRANSPOSE(G34:I34)/COUNTIF($A$2:$A$103,F30))</f>
+        <v>0.56000000000000005</v>
       </c>
       <c r="N32" s="57" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="str">
-        <f>'Human Grading'!A34</f>
-        <v>Composite State</v>
+        <f>'Human Grading'!A33</f>
+        <v>Action</v>
       </c>
       <c r="B33" s="5" t="str">
-        <f>'Human Grading'!B34</f>
-        <v>Baking</v>
+        <f>'Human Grading'!B33</f>
+        <v>setCourseTimes()</v>
       </c>
       <c r="C33" s="5">
         <f>'Human Grading'!C33</f>
@@ -20706,20 +20720,20 @@
         <v>1</v>
       </c>
       <c r="G33" s="58">
-        <f>COUNTIFS($A$2:$A$47,$F$30,$C$2:$C$47,$F33,$D$2:$D$47,G$30) + MAX(C50-D50,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$30,$C$2:$C$49,$F33,$D$2:$D$49,G$30) + MAX(C52-D52,0)</f>
         <v>0</v>
       </c>
       <c r="H33" s="59">
-        <f>COUNTIFS($A$2:$A$91,$F$30,$C$2:$C$91,$F33,$D$2:$D$91,H$30)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$30,$C$2:$C$93,$F33,$D$2:$D$93,H$30)</f>
         <v>0</v>
       </c>
       <c r="I33" s="60">
-        <f>COUNTIFS($A$2:$A$47,$F$30,$C$2:$C$47,$F33,$D$2:$D$47,I$30) + MIN(C50,D50)</f>
-        <v>4</v>
+        <f>COUNTIFS($A$2:$A$49,$F$30,$C$2:$C$49,$F33,$D$2:$D$49,I$30) + MIN(C52,D52)</f>
+        <v>3</v>
       </c>
       <c r="J33" s="14">
-        <f t="shared" si="16"/>
-        <v>4</v>
+        <f t="shared" si="8"/>
+        <v>3</v>
       </c>
       <c r="K33" s="14"/>
       <c r="L33" s="55" t="s">
@@ -20727,7 +20741,7 @@
       </c>
       <c r="M33" s="58">
         <f>(M31-M32)/(1-M32)</f>
-        <v>1</v>
+        <v>0.54545454545454553</v>
       </c>
       <c r="N33" s="60" t="s">
         <v>142</v>
@@ -20735,12 +20749,12 @@
     </row>
     <row r="34" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="5" t="str">
-        <f>'Human Grading'!A35</f>
-        <v>State</v>
+        <f>'Human Grading'!A34</f>
+        <v>Composite State</v>
       </c>
       <c r="B34" s="5" t="str">
-        <f>'Human Grading'!B35</f>
-        <v>Initial state</v>
+        <f>'Human Grading'!B34</f>
+        <v>Baking</v>
       </c>
       <c r="C34" s="5">
         <f>'Human Grading'!C34</f>
@@ -20755,15 +20769,15 @@
         <v>143</v>
       </c>
       <c r="G34" s="14">
-        <f t="shared" ref="G34:I34" si="18">SUM(G31:G33)</f>
+        <f t="shared" ref="G34:I34" si="9">SUM(G31:G33)</f>
         <v>1</v>
       </c>
       <c r="H34" s="14">
-        <f t="shared" si="18"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I34" s="14">
-        <f t="shared" si="18"/>
+        <f t="shared" si="9"/>
         <v>4</v>
       </c>
       <c r="J34" s="14"/>
@@ -20772,61 +20786,61 @@
     </row>
     <row r="35" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="5" t="str">
+        <f>'Human Grading'!A35</f>
+        <v>State</v>
+      </c>
+      <c r="B35" s="5" t="str">
+        <f>'Human Grading'!B35</f>
+        <v>Initial state</v>
+      </c>
+      <c r="C35" s="5">
+        <f>'Human Grading'!C35</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="5">
+        <f>'LLM Grading'!C35</f>
+        <v>1</v>
+      </c>
+      <c r="E35" s="44"/>
+    </row>
+    <row r="36" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="str">
         <f>'Human Grading'!A36</f>
         <v>State</v>
       </c>
-      <c r="B35" s="5" t="str">
+      <c r="B36" s="5" t="str">
         <f>'Human Grading'!B36</f>
         <v>Kneading</v>
       </c>
-      <c r="C35" s="5">
-        <f>'Human Grading'!C35</f>
-        <v>1</v>
-      </c>
-      <c r="D35" s="5">
-        <f>'LLM Grading'!C35</f>
-        <v>1</v>
-      </c>
-      <c r="E35" s="44"/>
-    </row>
-    <row r="36" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="5" t="str">
+      <c r="C36" s="5">
+        <f>'Human Grading'!C36</f>
+        <v>1</v>
+      </c>
+      <c r="D36" s="5">
+        <f>'LLM Grading'!C36</f>
+        <v>1</v>
+      </c>
+      <c r="E36" s="44"/>
+      <c r="F36" s="68" t="s">
+        <v>152</v>
+      </c>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
+      <c r="I36" s="69"/>
+      <c r="L36" s="72" t="s">
+        <v>153</v>
+      </c>
+      <c r="M36" s="73"/>
+      <c r="N36" s="73"/>
+    </row>
+    <row r="37" spans="1:14" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="5" t="str">
         <f>'Human Grading'!A37</f>
         <v>Action</v>
       </c>
-      <c r="B36" s="5" t="str">
+      <c r="B37" s="5" t="str">
         <f>'Human Grading'!B37</f>
         <v>startKneading()</v>
-      </c>
-      <c r="C36" s="5">
-        <f>'Human Grading'!C36</f>
-        <v>1</v>
-      </c>
-      <c r="D36" s="5">
-        <f>'LLM Grading'!C36</f>
-        <v>1</v>
-      </c>
-      <c r="E36" s="44"/>
-      <c r="F36" s="69" t="s">
-        <v>152</v>
-      </c>
-      <c r="G36" s="70"/>
-      <c r="H36" s="70"/>
-      <c r="I36" s="70"/>
-      <c r="L36" s="71" t="s">
-        <v>153</v>
-      </c>
-      <c r="M36" s="72"/>
-      <c r="N36" s="72"/>
-    </row>
-    <row r="37" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="5" t="str">
-        <f>'Human Grading'!A38</f>
-        <v>Action</v>
-      </c>
-      <c r="B37" s="5" t="str">
-        <f>'Human Grading'!B38</f>
-        <v>stopKneading()</v>
       </c>
       <c r="C37" s="5">
         <f>'Human Grading'!C37</f>
@@ -20865,12 +20879,12 @@
     </row>
     <row r="38" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="5" t="str">
-        <f>'Human Grading'!A39</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A38</f>
+        <v>Action</v>
       </c>
       <c r="B38" s="5" t="str">
-        <f>'Human Grading'!B39</f>
-        <v>baking initial state =&gt; kneading</v>
+        <f>'Human Grading'!B38</f>
+        <v>stopKneading()</v>
       </c>
       <c r="C38" s="5">
         <f>'Human Grading'!C38</f>
@@ -20885,28 +20899,28 @@
         <v>0</v>
       </c>
       <c r="G38" s="52">
-        <f t="shared" ref="G38:H38" si="19">COUNTIFS($A$2:$A$91,$F$37,$C$2:$C$91,$F38,$D$2:$D$91,G$37)</f>
-        <v>2</v>
+        <f>COUNTIFS($A$2:$A$93,$F$37,$C$2:$C$93,$F38,$D$2:$D$93,G$37)</f>
+        <v>6</v>
       </c>
       <c r="H38" s="53">
-        <f t="shared" si="19"/>
+        <f>COUNTIFS($A$2:$A$93,$F$37,$C$2:$C$93,$F38,$D$2:$D$93,H$37)</f>
         <v>0</v>
       </c>
       <c r="I38" s="54">
-        <f>COUNTIFS($A$2:$A$47,$F$37,$C$2:$C$47,$F38,$D$2:$D$47,I$37)+MAX(D51-C51,0)</f>
-        <v>1</v>
+        <f>COUNTIFS($A$2:$A$49,$F$37,$C$2:$C$49,$F38,$D$2:$D$49,I$37)+MAX(D53-C53,0)</f>
+        <v>0</v>
       </c>
       <c r="J38" s="14">
-        <f t="shared" ref="J38:J40" si="20">SUM(G38:I38)</f>
-        <v>3</v>
+        <f t="shared" ref="J38:J40" si="10">SUM(G38:I38)</f>
+        <v>6</v>
       </c>
       <c r="K38" s="14"/>
       <c r="L38" s="55" t="s">
         <v>138</v>
       </c>
       <c r="M38" s="52">
-        <f>(G38+H39+I40)/COUNTIF($A$2:$A$101,F37)</f>
-        <v>0.81818181818181823</v>
+        <f>(G38+H39+I40)/COUNTIF($A$2:$A$103,F37)</f>
+        <v>0.90909090909090906</v>
       </c>
       <c r="N38" s="54" t="s">
         <v>139</v>
@@ -20914,12 +20928,12 @@
     </row>
     <row r="39" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="5" t="str">
-        <f>'Human Grading'!A40</f>
+        <f>'Human Grading'!A39</f>
         <v>Transition</v>
       </c>
       <c r="B39" s="5" t="str">
-        <f>'Human Grading'!B40</f>
-        <v>kneading =&gt; rising</v>
+        <f>'Human Grading'!B39</f>
+        <v>baking initial state =&gt; kneading</v>
       </c>
       <c r="C39" s="5">
         <f>'Human Grading'!C39</f>
@@ -20934,19 +20948,19 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="56">
-        <f t="shared" ref="G39:I39" si="21">COUNTIFS($A$2:$A$91,$F$37,$C$2:$C$91,$F39,$D$2:$D$91,G$37)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$37,$C$2:$C$93,$F39,$D$2:$D$93,G$37)</f>
         <v>0</v>
       </c>
       <c r="H39" s="14">
-        <f t="shared" si="21"/>
+        <f>COUNTIFS($A$2:$A$93,$F$37,$C$2:$C$93,$F39,$D$2:$D$93,H$37)</f>
         <v>0</v>
       </c>
       <c r="I39" s="57">
-        <f t="shared" si="21"/>
+        <f>COUNTIFS($A$2:$A$93,$F$37,$C$2:$C$93,$F39,$D$2:$D$93,I$37)</f>
         <v>0</v>
       </c>
       <c r="J39" s="14">
-        <f t="shared" si="20"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="K39" s="14"/>
@@ -20954,21 +20968,21 @@
         <v>140</v>
       </c>
       <c r="M39" s="56">
-        <f t="array" ref="M39">SUMPRODUCT(J38:J40/COUNTIF($A$2:$A$101,F37), TRANSPOSE(G41:I41)/COUNTIF($A$2:$A$101,F37))</f>
-        <v>0.60330578512396693</v>
+        <f t="array" ref="M39">SUMPRODUCT(J38:J40/COUNTIF($A$2:$A$103,F37), TRANSPOSE(G41:I41)/COUNTIF($A$2:$A$103,F37))</f>
+        <v>0.51239669421487599</v>
       </c>
       <c r="N39" s="57" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="str">
-        <f>'Human Grading'!A41</f>
-        <v>State</v>
+        <f>'Human Grading'!A40</f>
+        <v>Transition</v>
       </c>
       <c r="B40" s="5" t="str">
-        <f>'Human Grading'!B41</f>
-        <v>Rising</v>
+        <f>'Human Grading'!B40</f>
+        <v>kneading =&gt; rising</v>
       </c>
       <c r="C40" s="5">
         <f>'Human Grading'!C40</f>
@@ -20983,20 +20997,20 @@
         <v>1</v>
       </c>
       <c r="G40" s="58">
-        <f>COUNTIFS($A$2:$A$47,$F$37,$C$2:$C$47,$F40,$D$2:$D$47,G$37)+MAX(C51-D51,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$37,$C$2:$C$49,$F40,$D$2:$D$49,G$37)+MAX(C53-D53,0)</f>
         <v>1</v>
       </c>
       <c r="H40" s="59">
-        <f>COUNTIFS($A$2:$A$91,$F$37,$C$2:$C$91,$F40,$D$2:$D$91,H$37)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$37,$C$2:$C$93,$F40,$D$2:$D$93,H$37)</f>
         <v>0</v>
       </c>
       <c r="I40" s="60">
-        <f>COUNTIFS($A$2:$A$47,$F$37,$C$2:$C$47,$F40,$D$2:$D$47,I$37) + MIN(C51,D51)</f>
-        <v>7</v>
+        <f>COUNTIFS($A$2:$A$49,$F$37,$C$2:$C$49,$F40,$D$2:$D$49,I$37) + MIN(C53,D53)</f>
+        <v>4</v>
       </c>
       <c r="J40" s="14">
-        <f t="shared" si="20"/>
-        <v>8</v>
+        <f t="shared" si="10"/>
+        <v>5</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="55" t="s">
@@ -21004,7 +21018,7 @@
       </c>
       <c r="M40" s="58">
         <f>(M38-M39)/(1-M39)</f>
-        <v>0.54166666666666685</v>
+        <v>0.81355932203389825</v>
       </c>
       <c r="N40" s="60" t="s">
         <v>142</v>
@@ -21012,12 +21026,12 @@
     </row>
     <row r="41" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="5" t="str">
-        <f>'Human Grading'!A42</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A41</f>
+        <v>State</v>
       </c>
       <c r="B41" s="5" t="str">
-        <f>'Human Grading'!B42</f>
-        <v>rising =&gt; baking</v>
+        <f>'Human Grading'!B41</f>
+        <v>Rising</v>
       </c>
       <c r="C41" s="5">
         <f>'Human Grading'!C41</f>
@@ -21032,16 +21046,16 @@
         <v>143</v>
       </c>
       <c r="G41" s="14">
-        <f t="shared" ref="G41:I41" si="22">SUM(G38:G40)</f>
-        <v>3</v>
+        <f t="shared" ref="G41:I41" si="11">SUM(G38:G40)</f>
+        <v>7</v>
       </c>
       <c r="H41" s="14">
-        <f t="shared" si="22"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="I41" s="14">
-        <f t="shared" si="22"/>
-        <v>8</v>
+        <f t="shared" si="11"/>
+        <v>4</v>
       </c>
       <c r="J41" s="14"/>
       <c r="L41" s="14"/>
@@ -21049,61 +21063,61 @@
     </row>
     <row r="42" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="5" t="str">
+        <f>'Human Grading'!A42</f>
+        <v>Transition</v>
+      </c>
+      <c r="B42" s="5" t="str">
+        <f>'Human Grading'!B42</f>
+        <v>rising =&gt; baking</v>
+      </c>
+      <c r="C42" s="5">
+        <f>'Human Grading'!C42</f>
+        <v>1</v>
+      </c>
+      <c r="D42" s="5">
+        <f>'LLM Grading'!C42</f>
+        <v>1</v>
+      </c>
+      <c r="E42" s="44"/>
+    </row>
+    <row r="43" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="5" t="str">
         <f>'Human Grading'!A43</f>
         <v>State</v>
       </c>
-      <c r="B42" s="5" t="str">
+      <c r="B43" s="5" t="str">
         <f>'Human Grading'!B43</f>
         <v>Baking</v>
       </c>
-      <c r="C42" s="5">
-        <f>'Human Grading'!C42</f>
-        <v>1</v>
-      </c>
-      <c r="D42" s="5">
-        <f>'LLM Grading'!C42</f>
-        <v>1</v>
-      </c>
-      <c r="E42" s="44"/>
-    </row>
-    <row r="43" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="5" t="str">
+      <c r="C43" s="5">
+        <f>'Human Grading'!C43</f>
+        <v>1</v>
+      </c>
+      <c r="D43" s="5">
+        <f>'LLM Grading'!C43</f>
+        <v>1</v>
+      </c>
+      <c r="E43" s="44"/>
+      <c r="F43" s="68" t="s">
+        <v>154</v>
+      </c>
+      <c r="G43" s="69"/>
+      <c r="H43" s="69"/>
+      <c r="I43" s="69"/>
+      <c r="L43" s="72" t="s">
+        <v>155</v>
+      </c>
+      <c r="M43" s="73"/>
+      <c r="N43" s="73"/>
+    </row>
+    <row r="44" spans="1:14" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="str">
         <f>'Human Grading'!A44</f>
         <v>Action</v>
       </c>
-      <c r="B43" s="5" t="str">
+      <c r="B44" s="5" t="str">
         <f>'Human Grading'!B44</f>
         <v>heat()</v>
-      </c>
-      <c r="C43" s="5">
-        <f>'Human Grading'!C43</f>
-        <v>1</v>
-      </c>
-      <c r="D43" s="5">
-        <f>'LLM Grading'!C43</f>
-        <v>1</v>
-      </c>
-      <c r="E43" s="44"/>
-      <c r="F43" s="69" t="s">
-        <v>154</v>
-      </c>
-      <c r="G43" s="70"/>
-      <c r="H43" s="70"/>
-      <c r="I43" s="70"/>
-      <c r="L43" s="71" t="s">
-        <v>155</v>
-      </c>
-      <c r="M43" s="72"/>
-      <c r="N43" s="72"/>
-    </row>
-    <row r="44" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A44" s="5" t="str">
-        <f>'Human Grading'!A45</f>
-        <v>Transition</v>
-      </c>
-      <c r="B44" s="5" t="str">
-        <f>'Human Grading'!B45</f>
-        <v>baking =&gt; warming</v>
       </c>
       <c r="C44" s="5">
         <f>'Human Grading'!C44</f>
@@ -21142,12 +21156,12 @@
     </row>
     <row r="45" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="5" t="str">
-        <f>'Human Grading'!A46</f>
-        <v>State</v>
+        <f>'Human Grading'!A45</f>
+        <v>Transition</v>
       </c>
       <c r="B45" s="5" t="str">
-        <f>'Human Grading'!B46</f>
-        <v>Warming</v>
+        <f>'Human Grading'!B45</f>
+        <v>baking =&gt; warming</v>
       </c>
       <c r="C45" s="5">
         <f>'Human Grading'!C45</f>
@@ -21162,28 +21176,28 @@
         <v>0</v>
       </c>
       <c r="G45" s="52">
-        <f t="shared" ref="G45:H45" si="23">COUNTIFS($A$2:$A$91,$F$44,$C$2:$C$91,$F45,$D$2:$D$91,G$44)</f>
-        <v>1</v>
+        <f>COUNTIFS($A$2:$A$93,$F$44,$C$2:$C$93,$F45,$D$2:$D$93,G$44)</f>
+        <v>2</v>
       </c>
       <c r="H45" s="53">
-        <f t="shared" si="23"/>
+        <f>COUNTIFS($A$2:$A$93,$F$44,$C$2:$C$93,$F45,$D$2:$D$93,H$44)</f>
         <v>0</v>
       </c>
       <c r="I45" s="54">
-        <f>COUNTIFS($A$2:$A$47,$F$44,$C$2:$C$47,$F45,$D$2:$D$47,I$44) + MAX(D54-C54,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$44,$C$2:$C$49,$F45,$D$2:$D$49,I$44) + MAX(D56-C56,0)</f>
         <v>0</v>
       </c>
       <c r="J45" s="14">
-        <f t="shared" ref="J45:J47" si="24">SUM(G45:I45)</f>
-        <v>1</v>
+        <f t="shared" ref="J45:J47" si="12">SUM(G45:I45)</f>
+        <v>2</v>
       </c>
       <c r="K45" s="14"/>
       <c r="L45" s="55" t="s">
         <v>138</v>
       </c>
       <c r="M45" s="52">
-        <f>(G45+H46+I47)/COUNTIF($A$2:$A$101,F44)</f>
-        <v>0.5</v>
+        <f>(G45+H46+I47)/COUNTIF($A$2:$A$103,F44)</f>
+        <v>1</v>
       </c>
       <c r="N45" s="54" t="s">
         <v>139</v>
@@ -21191,12 +21205,12 @@
     </row>
     <row r="46" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="5" t="str">
-        <f>'Human Grading'!A47</f>
-        <v>Action</v>
+        <f>'Human Grading'!A46</f>
+        <v>State</v>
       </c>
       <c r="B46" s="5" t="str">
-        <f>'Human Grading'!B47</f>
-        <v>warm()</v>
+        <f>'Human Grading'!B46</f>
+        <v>Warming</v>
       </c>
       <c r="C46" s="5">
         <f>'Human Grading'!C46</f>
@@ -21211,47 +21225,47 @@
         <v>0.5</v>
       </c>
       <c r="G46" s="56">
-        <f t="shared" ref="G46:I46" si="25">COUNTIFS($A$2:$A$91,$F$44,$C$2:$C$91,$F46,$D$2:$D$91,G$44)</f>
-        <v>1</v>
+        <f>COUNTIFS($A$2:$A$93,$F$44,$C$2:$C$93,$F46,$D$2:$D$93,G$44)</f>
+        <v>0</v>
       </c>
       <c r="H46" s="14">
-        <f t="shared" si="25"/>
+        <f>COUNTIFS($A$2:$A$93,$F$44,$C$2:$C$93,$F46,$D$2:$D$93,H$44)</f>
         <v>0</v>
       </c>
       <c r="I46" s="57">
-        <f t="shared" si="25"/>
+        <f>COUNTIFS($A$2:$A$93,$F$44,$C$2:$C$93,$F46,$D$2:$D$93,I$44)</f>
         <v>0</v>
       </c>
       <c r="J46" s="14">
-        <f t="shared" si="24"/>
-        <v>1</v>
+        <f t="shared" si="12"/>
+        <v>0</v>
       </c>
       <c r="K46" s="14"/>
       <c r="L46" s="55" t="s">
         <v>140</v>
       </c>
       <c r="M46" s="56">
-        <f t="array" ref="M46">SUMPRODUCT(J45:J47/COUNTIF($A$2:$A$101,F44), TRANSPOSE(G48:I48)/COUNTIF($A$2:$A$101,F44))</f>
-        <v>0.5</v>
+        <f t="array" ref="M46">SUMPRODUCT(J45:J47/COUNTIF($A$2:$A$103,F44), TRANSPOSE(G48:I48)/COUNTIF($A$2:$A$103,F44))</f>
+        <v>1</v>
       </c>
       <c r="N46" s="57" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="str">
-        <f>'Human Grading'!A48</f>
-        <v>Transition</v>
+        <f>'Human Grading'!A47</f>
+        <v>Action</v>
       </c>
       <c r="B47" s="5" t="str">
-        <f>'Human Grading'!B48</f>
-        <v>after 60min (warming =&gt; setup)</v>
-      </c>
-      <c r="C47" s="65">
+        <f>'Human Grading'!B47</f>
+        <v>warm()</v>
+      </c>
+      <c r="C47" s="5">
         <f>'Human Grading'!C47</f>
         <v>1</v>
       </c>
-      <c r="D47" s="65">
+      <c r="D47" s="5">
         <f>'LLM Grading'!C47</f>
         <v>1</v>
       </c>
@@ -21260,47 +21274,47 @@
         <v>1</v>
       </c>
       <c r="G47" s="58">
-        <f>COUNTIFS($A$2:$A$47,$F$44,$C$2:$C$47,$F47,$D$2:$D$47,G$44) + MAX(C54-D54,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$44,$C$2:$C$49,$F47,$D$2:$D$49,G$44) + MAX(C56-D56,0)</f>
         <v>0</v>
       </c>
       <c r="H47" s="59">
-        <f>COUNTIFS($A$2:$A$91,$F$44,$C$2:$C$91,$F47,$D$2:$D$91,H$44)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$44,$C$2:$C$93,$F47,$D$2:$D$93,H$44)</f>
         <v>0</v>
       </c>
       <c r="I47" s="60">
-        <f>COUNTIFS($A$2:$A$47,$F$44,$C$2:$C$47,$F47,$D$2:$D$47,I$44) + MIN(C54,D54)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$44,$C$2:$C$49,$F47,$D$2:$D$49,I$44) + MIN(C56,D56)</f>
         <v>0</v>
       </c>
       <c r="J47" s="14">
-        <f t="shared" si="24"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="K47" s="14"/>
       <c r="L47" s="55" t="s">
         <v>129</v>
       </c>
-      <c r="M47" s="58">
+      <c r="M47" s="58" t="e">
         <f>(M45-M46)/(1-M46)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N47" s="60" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A48" s="12" t="str">
-        <f>'Human Grading'!A50</f>
-        <v>State</v>
-      </c>
-      <c r="B48" s="12" t="str">
-        <f>'Human Grading'!B50</f>
-        <v>additional elements</v>
-      </c>
-      <c r="C48" s="12">
+      <c r="A48" s="5" t="str">
+        <f>'Human Grading'!A48</f>
+        <v>Transition</v>
+      </c>
+      <c r="B48" s="5" t="str">
+        <f>'Human Grading'!B48</f>
+        <v>after 60min (warming =&gt; setup)</v>
+      </c>
+      <c r="C48" s="5">
         <f>'Human Grading'!C48</f>
         <v>1</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="5">
         <f>'LLM Grading'!C48</f>
         <v>1</v>
       </c>
@@ -21309,15 +21323,15 @@
         <v>143</v>
       </c>
       <c r="G48" s="14">
-        <f t="shared" ref="G48:I48" si="26">SUM(G45:G47)</f>
+        <f t="shared" ref="G48:I48" si="13">SUM(G45:G47)</f>
         <v>2</v>
       </c>
       <c r="H48" s="14">
-        <f t="shared" si="26"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="I48" s="14">
-        <f t="shared" si="26"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="J48" s="14"/>
@@ -21326,60 +21340,60 @@
     </row>
     <row r="49" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="5" t="str">
+        <f>'Human Grading'!A49</f>
+        <v>Transition</v>
+      </c>
+      <c r="B49" s="5" t="str">
+        <f>'Human Grading'!B49</f>
+        <v>baking =&gt; setup</v>
+      </c>
+      <c r="C49" s="5">
+        <f>'Human Grading'!C49</f>
+        <v>1</v>
+      </c>
+      <c r="D49" s="5">
+        <f>'LLM Grading'!C49</f>
+        <v>1</v>
+      </c>
+      <c r="E49" s="44"/>
+    </row>
+    <row r="50" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="5" t="str">
+        <f>'Human Grading'!A50</f>
+        <v>State</v>
+      </c>
+      <c r="B50" s="5" t="str">
+        <f>'Human Grading'!B50</f>
+        <v>additional elements</v>
+      </c>
+      <c r="C50" s="5">
+        <f>'Human Grading'!C50</f>
+        <v>0</v>
+      </c>
+      <c r="D50" s="5">
+        <f>'LLM Grading'!C50</f>
+        <v>0</v>
+      </c>
+      <c r="E50" s="44"/>
+      <c r="F50" s="68" t="s">
+        <v>156</v>
+      </c>
+      <c r="G50" s="69"/>
+      <c r="H50" s="69"/>
+      <c r="I50" s="69"/>
+      <c r="L50" s="72" t="s">
+        <v>157</v>
+      </c>
+      <c r="M50" s="73"/>
+      <c r="N50" s="73"/>
+    </row>
+    <row r="51" spans="1:14" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="5" t="str">
         <f>'Human Grading'!A51</f>
         <v>Transition</v>
       </c>
-      <c r="B49" s="5" t="str">
+      <c r="B51" s="5" t="str">
         <f>'Human Grading'!B51</f>
-        <v>additional elements</v>
-      </c>
-      <c r="C49" s="5">
-        <f>'Human Grading'!C49</f>
-        <v>1</v>
-      </c>
-      <c r="D49" s="5">
-        <f>'LLM Grading'!C49</f>
-        <v>1</v>
-      </c>
-      <c r="E49" s="44"/>
-    </row>
-    <row r="50" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A50" s="5" t="str">
-        <f>'Human Grading'!A52</f>
-        <v>Guard</v>
-      </c>
-      <c r="B50" s="5" t="str">
-        <f>'Human Grading'!B52</f>
-        <v>additional elements</v>
-      </c>
-      <c r="C50" s="5">
-        <f>'Human Grading'!C50</f>
-        <v>0</v>
-      </c>
-      <c r="D50" s="5">
-        <f>'LLM Grading'!C50</f>
-        <v>0</v>
-      </c>
-      <c r="E50" s="44"/>
-      <c r="F50" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="G50" s="70"/>
-      <c r="H50" s="70"/>
-      <c r="I50" s="70"/>
-      <c r="L50" s="71" t="s">
-        <v>157</v>
-      </c>
-      <c r="M50" s="72"/>
-      <c r="N50" s="72"/>
-    </row>
-    <row r="51" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A51" s="5" t="str">
-        <f>'Human Grading'!A53</f>
-        <v>Action</v>
-      </c>
-      <c r="B51" s="5" t="str">
-        <f>'Human Grading'!B53</f>
         <v>additional elements</v>
       </c>
       <c r="C51" s="5">
@@ -21419,11 +21433,11 @@
     </row>
     <row r="52" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="5" t="str">
-        <f>'Human Grading'!A54</f>
-        <v>Composite State</v>
+        <f>'Human Grading'!A52</f>
+        <v>Guard</v>
       </c>
       <c r="B52" s="5" t="str">
-        <f>'Human Grading'!B54</f>
+        <f>'Human Grading'!B52</f>
         <v>additional elements</v>
       </c>
       <c r="C52" s="5">
@@ -21439,19 +21453,19 @@
         <v>0</v>
       </c>
       <c r="G52" s="52">
-        <f t="shared" ref="G52:H52" si="27">COUNTIFS($A$2:$A$91,$F$51,$C$2:$C$91,$F52,$D$2:$D$91,G$51)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$51,$C$2:$C$93,$F52,$D$2:$D$93,G$51)</f>
         <v>1</v>
       </c>
       <c r="H52" s="53">
-        <f t="shared" si="27"/>
+        <f>COUNTIFS($A$2:$A$93,$F$51,$C$2:$C$93,$F52,$D$2:$D$93,H$51)</f>
         <v>0</v>
       </c>
       <c r="I52" s="54">
-        <f>COUNTIFS($A$2:$A$47,$F$51,$C$2:$C$47,$F52,$D$2:$D$47,I$51)+MAX(D53-C53,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$51,$C$2:$C$49,$F52,$D$2:$D$49,I$51)+MAX(D55-C55,0)</f>
         <v>0</v>
       </c>
       <c r="J52" s="14">
-        <f t="shared" ref="J52:J54" si="28">SUM(G52:I52)</f>
+        <f t="shared" ref="J52:J54" si="14">SUM(G52:I52)</f>
         <v>1</v>
       </c>
       <c r="K52" s="14"/>
@@ -21459,7 +21473,7 @@
         <v>138</v>
       </c>
       <c r="M52" s="52">
-        <f>(G52+H53+I54)/COUNTIF($A$2:$A$101,F51)</f>
+        <f>(G52+H53+I54)/COUNTIF($A$2:$A$103,F51)</f>
         <v>1</v>
       </c>
       <c r="N52" s="54" t="s">
@@ -21468,11 +21482,11 @@
     </row>
     <row r="53" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="5" t="str">
-        <f>'Human Grading'!A55</f>
-        <v>Region</v>
+        <f>'Human Grading'!A53</f>
+        <v>Action</v>
       </c>
       <c r="B53" s="5" t="str">
-        <f>'Human Grading'!B55</f>
+        <f>'Human Grading'!B53</f>
         <v>additional elements</v>
       </c>
       <c r="C53" s="5">
@@ -21488,19 +21502,19 @@
         <v>0.5</v>
       </c>
       <c r="G53" s="56">
-        <f t="shared" ref="G53:I53" si="29">COUNTIFS($A$2:$A$91,$F$51,$C$2:$C$91,$F53,$D$2:$D$91,G$51)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$51,$C$2:$C$93,$F53,$D$2:$D$93,G$51)</f>
         <v>0</v>
       </c>
       <c r="H53" s="14">
-        <f t="shared" si="29"/>
+        <f>COUNTIFS($A$2:$A$93,$F$51,$C$2:$C$93,$F53,$D$2:$D$93,H$51)</f>
         <v>0</v>
       </c>
       <c r="I53" s="57">
-        <f t="shared" si="29"/>
+        <f>COUNTIFS($A$2:$A$93,$F$51,$C$2:$C$93,$F53,$D$2:$D$93,I$51)</f>
         <v>0</v>
       </c>
       <c r="J53" s="14">
-        <f t="shared" si="28"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="K53" s="14"/>
@@ -21508,20 +21522,20 @@
         <v>140</v>
       </c>
       <c r="M53" s="56">
-        <f t="array" ref="M53">SUMPRODUCT(J52:J54/COUNTIF($A$2:$A$101,F51), TRANSPOSE(G55:I55)/COUNTIF($A$2:$A$101,F51))</f>
+        <f t="array" ref="M53">SUMPRODUCT(J52:J54/COUNTIF($A$2:$A$103,F51), TRANSPOSE(G55:I55)/COUNTIF($A$2:$A$103,F51))</f>
         <v>1</v>
       </c>
       <c r="N53" s="57" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="str">
-        <f>'Human Grading'!A56</f>
-        <v>History State</v>
+        <f>'Human Grading'!A54</f>
+        <v>Composite State</v>
       </c>
       <c r="B54" s="5" t="str">
-        <f>'Human Grading'!B56</f>
+        <f>'Human Grading'!B54</f>
         <v>additional elements</v>
       </c>
       <c r="C54" s="5">
@@ -21537,19 +21551,19 @@
         <v>1</v>
       </c>
       <c r="G54" s="58">
-        <f>COUNTIFS($A$2:$A$47,$F$51,$C$2:$C$47,$F54,$D$2:$D$47,G$51) + MAX(C53-D53,0)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$51,$C$2:$C$49,$F54,$D$2:$D$49,G$51) + MAX(C55-D55,0)</f>
         <v>0</v>
       </c>
       <c r="H54" s="59">
-        <f>COUNTIFS($A$2:$A$91,$F$51,$C$2:$C$91,$F54,$D$2:$D$91,H$51)</f>
+        <f>COUNTIFS($A$2:$A$93,$F$51,$C$2:$C$93,$F54,$D$2:$D$93,H$51)</f>
         <v>0</v>
       </c>
       <c r="I54" s="60">
-        <f>COUNTIFS($A$2:$A$47,$F$51,$C$2:$C$47,$F54,$D$2:$D$47,I$51)+MIN(C53,D53)</f>
+        <f>COUNTIFS($A$2:$A$49,$F$51,$C$2:$C$49,$F54,$D$2:$D$49,I$51)+MIN(C55,D55)</f>
         <v>0</v>
       </c>
       <c r="J54" s="14">
-        <f t="shared" si="28"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="K54" s="14"/>
@@ -21565,24 +21579,36 @@
       </c>
     </row>
     <row r="55" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A55" s="45"/>
-      <c r="B55" s="66"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
+      <c r="A55" s="5" t="str">
+        <f>'Human Grading'!A55</f>
+        <v>Region</v>
+      </c>
+      <c r="B55" s="5" t="str">
+        <f>'Human Grading'!B55</f>
+        <v>additional elements</v>
+      </c>
+      <c r="C55" s="5">
+        <f>'Human Grading'!C55</f>
+        <v>0</v>
+      </c>
+      <c r="D55" s="5">
+        <f>'LLM Grading'!C55</f>
+        <v>0</v>
+      </c>
       <c r="E55" s="44"/>
       <c r="F55" s="61" t="s">
         <v>143</v>
       </c>
       <c r="G55" s="14">
-        <f t="shared" ref="G55:I55" si="30">SUM(G52:G54)</f>
+        <f t="shared" ref="G55:I55" si="15">SUM(G52:G54)</f>
         <v>1</v>
       </c>
       <c r="H55" s="14">
-        <f t="shared" si="30"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="I55" s="14">
-        <f t="shared" si="30"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="J55" s="14"/>
@@ -21590,10 +21616,22 @@
       <c r="M55" s="62"/>
     </row>
     <row r="56" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A56" s="45"/>
-      <c r="B56" s="66"/>
-      <c r="C56" s="44"/>
-      <c r="D56" s="44"/>
+      <c r="A56" s="5" t="str">
+        <f>'Human Grading'!A56</f>
+        <v>History State</v>
+      </c>
+      <c r="B56" s="5" t="str">
+        <f>'Human Grading'!B56</f>
+        <v>additional elements</v>
+      </c>
+      <c r="C56" s="5">
+        <f>'Human Grading'!C56</f>
+        <v>0</v>
+      </c>
+      <c r="D56" s="5">
+        <f>'LLM Grading'!C56</f>
+        <v>0</v>
+      </c>
       <c r="E56" s="44"/>
     </row>
     <row r="57" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -21738,32 +21776,42 @@
       <c r="D77" s="44"/>
     </row>
     <row r="78" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A78" s="45"/>
       <c r="B78" s="66"/>
+      <c r="C78" s="44"/>
       <c r="D78" s="44"/>
     </row>
     <row r="79" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" s="45"/>
       <c r="B79" s="66"/>
+      <c r="C79" s="44"/>
       <c r="D79" s="44"/>
     </row>
     <row r="80" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B80" s="66"/>
       <c r="D80" s="44"/>
     </row>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="81" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B81" s="66"/>
+      <c r="D81" s="44"/>
+    </row>
+    <row r="82" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D82" s="44"/>
+    </row>
+    <row r="83" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="84" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="85" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="86" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="87" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="88" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="89" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="90" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="91" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="92" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="93" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="94" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="95" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="96" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -22670,6 +22718,12 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="L15:N15"/>
     <mergeCell ref="L22:N22"/>
     <mergeCell ref="F50:I50"/>
     <mergeCell ref="L50:N50"/>
@@ -22680,12 +22734,6 @@
     <mergeCell ref="L36:N36"/>
     <mergeCell ref="F43:I43"/>
     <mergeCell ref="L43:N43"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="L15:N15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -22726,25 +22774,25 @@
       <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="73" t="s">
+      <c r="C1" s="67" t="s">
         <v>166</v>
       </c>
-      <c r="D1" s="73" t="s">
+      <c r="D1" s="67" t="s">
         <v>60</v>
       </c>
       <c r="E1" s="44"/>
-      <c r="F1" s="69" t="s">
+      <c r="F1" s="68" t="s">
         <v>128</v>
       </c>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="L1" s="69" t="s">
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="L1" s="68" t="s">
         <v>158</v>
       </c>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
     </row>
     <row r="2" spans="1:24" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="str">
@@ -23148,12 +23196,12 @@
         <v>0</v>
       </c>
       <c r="E8" s="44"/>
-      <c r="F8" s="69" t="s">
+      <c r="F8" s="68" t="s">
         <v>144</v>
       </c>
-      <c r="G8" s="70"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="70"/>
+      <c r="G8" s="69"/>
+      <c r="H8" s="69"/>
+      <c r="I8" s="69"/>
     </row>
     <row r="9" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="5" t="str">
@@ -23543,12 +23591,12 @@
         <v>0</v>
       </c>
       <c r="E15" s="44"/>
-      <c r="F15" s="69" t="s">
+      <c r="F15" s="68" t="s">
         <v>146</v>
       </c>
-      <c r="G15" s="70"/>
-      <c r="H15" s="70"/>
-      <c r="I15" s="70"/>
+      <c r="G15" s="69"/>
+      <c r="H15" s="69"/>
+      <c r="I15" s="69"/>
     </row>
     <row r="16" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="5" t="str">
@@ -23938,12 +23986,12 @@
         <v>1</v>
       </c>
       <c r="E22" s="44"/>
-      <c r="F22" s="69" t="s">
+      <c r="F22" s="68" t="s">
         <v>148</v>
       </c>
-      <c r="G22" s="70"/>
-      <c r="H22" s="70"/>
-      <c r="I22" s="70"/>
+      <c r="G22" s="69"/>
+      <c r="H22" s="69"/>
+      <c r="I22" s="69"/>
     </row>
     <row r="23" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="5" t="str">
@@ -24333,12 +24381,12 @@
         <v>1</v>
       </c>
       <c r="E29" s="44"/>
-      <c r="F29" s="69" t="s">
+      <c r="F29" s="68" t="s">
         <v>150</v>
       </c>
-      <c r="G29" s="70"/>
-      <c r="H29" s="70"/>
-      <c r="I29" s="70"/>
+      <c r="G29" s="69"/>
+      <c r="H29" s="69"/>
+      <c r="I29" s="69"/>
     </row>
     <row r="30" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="5" t="str">
@@ -24728,12 +24776,12 @@
         <v>1</v>
       </c>
       <c r="E36" s="44"/>
-      <c r="F36" s="69" t="s">
+      <c r="F36" s="68" t="s">
         <v>152</v>
       </c>
-      <c r="G36" s="70"/>
-      <c r="H36" s="70"/>
-      <c r="I36" s="70"/>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
+      <c r="I36" s="69"/>
     </row>
     <row r="37" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="5" t="str">
@@ -25123,12 +25171,12 @@
         <v>1</v>
       </c>
       <c r="E43" s="44"/>
-      <c r="F43" s="69" t="s">
+      <c r="F43" s="68" t="s">
         <v>154</v>
       </c>
-      <c r="G43" s="70"/>
-      <c r="H43" s="70"/>
-      <c r="I43" s="70"/>
+      <c r="G43" s="69"/>
+      <c r="H43" s="69"/>
+      <c r="I43" s="69"/>
     </row>
     <row r="44" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="5" t="str">
@@ -25518,12 +25566,12 @@
         <v>0</v>
       </c>
       <c r="E50" s="44"/>
-      <c r="F50" s="69" t="s">
+      <c r="F50" s="68" t="s">
         <v>156</v>
       </c>
-      <c r="G50" s="70"/>
-      <c r="H50" s="70"/>
-      <c r="I50" s="70"/>
+      <c r="G50" s="69"/>
+      <c r="H50" s="69"/>
+      <c r="I50" s="69"/>
     </row>
     <row r="51" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="5" t="str">

</xml_diff>